<commit_message>
feat: add Excel import root parent selection and WBS fallback
</commit_message>
<xml_diff>
--- a/data_sources/templates/openproject template.xlsx
+++ b/data_sources/templates/openproject template.xlsx
@@ -454,7 +454,7 @@
     <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
     <ns0:pageSetUpPr/>
   </ns0:sheetPr>
-  <ns0:dimension ref="A1:J1"/>
+  <ns0:dimension ref="A1:H1"/>
   <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <ns0:cols>
     <ns0:col width="83" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -501,16 +501,6 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="H1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Resource_Names</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="I1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Priority</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="J1" t="inlineStr">
         <ns0:is>
           <ns0:t>Type</ns0:t>
         </ns0:is>

</xml_diff>